<commit_message>
rm interpretation frm pb profile 7df15491d78c199a1c9bb56f14affd9107e365b6
</commit_message>
<xml_diff>
--- a/ig/nr-rm-interpretation-binding/StructureDefinition-fr-core-observation-bp.xlsx
+++ b/ig/nr-rm-interpretation-binding/StructureDefinition-fr-core-observation-bp.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6003" uniqueCount="682">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6006" uniqueCount="681">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-10-09T10:17:35+00:00</t>
+    <t>2023-10-09T10:19:35+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1955,9 +1955,6 @@
   </si>
   <si>
     <t>Observation.component:SystolicBP.interpretation</t>
-  </si>
-  <si>
-    <t>http://www.interopsante.org/fhir/structuredefinition/observation/fr-core-obervation-interpretation</t>
   </si>
   <si>
     <t>Observation.component:SystolicBP.referenceRange</t>
@@ -2484,7 +2481,7 @@
     <col min="23" max="23" width="1.04296875" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="10.53125" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="63.70703125" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="90.3359375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="65.33203125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="1.04296875" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="26.1796875" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="42.03515625" customWidth="true" bestFit="true"/>
@@ -15023,9 +15020,11 @@
       <c r="X104" t="s" s="2">
         <v>257</v>
       </c>
-      <c r="Y104" s="2"/>
+      <c r="Y104" t="s" s="2">
+        <v>375</v>
+      </c>
       <c r="Z104" t="s" s="2">
-        <v>620</v>
+        <v>376</v>
       </c>
       <c r="AA104" t="s" s="2">
         <v>38</v>
@@ -15078,7 +15077,7 @@
     </row>
     <row r="105" hidden="true">
       <c r="A105" t="s" s="2">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B105" t="s" s="2">
         <v>528</v>
@@ -15200,13 +15199,13 @@
     </row>
     <row r="106" hidden="true">
       <c r="A106" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B106" t="s" s="2">
         <v>496</v>
       </c>
       <c r="C106" t="s" s="2">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D106" t="s" s="2">
         <v>38</v>
@@ -15231,10 +15230,10 @@
         <v>426</v>
       </c>
       <c r="L106" t="s" s="2">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="M106" t="s" s="2">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="N106" t="s" s="2">
         <v>499</v>
@@ -15324,7 +15323,7 @@
     </row>
     <row r="107" hidden="true">
       <c r="A107" t="s" s="2">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B107" t="s" s="2">
         <v>505</v>
@@ -15442,7 +15441,7 @@
     </row>
     <row r="108" hidden="true">
       <c r="A108" t="s" s="2">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B108" t="s" s="2">
         <v>506</v>
@@ -15562,7 +15561,7 @@
     </row>
     <row r="109" hidden="true">
       <c r="A109" t="s" s="2">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B109" t="s" s="2">
         <v>507</v>
@@ -15684,7 +15683,7 @@
     </row>
     <row r="110" hidden="true">
       <c r="A110" t="s" s="2">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B110" t="s" s="2">
         <v>508</v>
@@ -15806,7 +15805,7 @@
     </row>
     <row r="111" hidden="true">
       <c r="A111" t="s" s="2">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B111" t="s" s="2">
         <v>539</v>
@@ -15924,7 +15923,7 @@
     </row>
     <row r="112" hidden="true">
       <c r="A112" t="s" s="2">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B112" t="s" s="2">
         <v>541</v>
@@ -16044,7 +16043,7 @@
     </row>
     <row r="113" hidden="true">
       <c r="A113" t="s" s="2">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B113" t="s" s="2">
         <v>543</v>
@@ -16073,10 +16072,10 @@
         <v>184</v>
       </c>
       <c r="L113" t="s" s="2">
+        <v>631</v>
+      </c>
+      <c r="M113" t="s" s="2">
         <v>632</v>
-      </c>
-      <c r="M113" t="s" s="2">
-        <v>633</v>
       </c>
       <c r="N113" t="s" s="2">
         <v>187</v>
@@ -16164,13 +16163,13 @@
     </row>
     <row r="114" hidden="true">
       <c r="A114" t="s" s="2">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B114" t="s" s="2">
         <v>543</v>
       </c>
       <c r="C114" t="s" s="2">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D114" t="s" s="2">
         <v>38</v>
@@ -16195,10 +16194,10 @@
         <v>184</v>
       </c>
       <c r="L114" t="s" s="2">
+        <v>631</v>
+      </c>
+      <c r="M114" t="s" s="2">
         <v>632</v>
-      </c>
-      <c r="M114" t="s" s="2">
-        <v>633</v>
       </c>
       <c r="N114" t="s" s="2">
         <v>187</v>
@@ -16288,7 +16287,7 @@
     </row>
     <row r="115" hidden="true">
       <c r="A115" t="s" s="2">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B115" t="s" s="2">
         <v>549</v>
@@ -16406,7 +16405,7 @@
     </row>
     <row r="116" hidden="true">
       <c r="A116" t="s" s="2">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B116" t="s" s="2">
         <v>551</v>
@@ -16526,7 +16525,7 @@
     </row>
     <row r="117" hidden="true">
       <c r="A117" t="s" s="2">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B117" t="s" s="2">
         <v>553</v>
@@ -16648,7 +16647,7 @@
     </row>
     <row r="118" hidden="true">
       <c r="A118" t="s" s="2">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B118" t="s" s="2">
         <v>555</v>
@@ -16768,7 +16767,7 @@
     </row>
     <row r="119" hidden="true">
       <c r="A119" t="s" s="2">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B119" t="s" s="2">
         <v>557</v>
@@ -16813,7 +16812,7 @@
       </c>
       <c r="Q119" s="2"/>
       <c r="R119" t="s" s="2">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="S119" t="s" s="2">
         <v>38</v>
@@ -16890,7 +16889,7 @@
     </row>
     <row r="120" hidden="true">
       <c r="A120" t="s" s="2">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B120" t="s" s="2">
         <v>560</v>
@@ -17012,7 +17011,7 @@
     </row>
     <row r="121" hidden="true">
       <c r="A121" t="s" s="2">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B121" t="s" s="2">
         <v>562</v>
@@ -17134,7 +17133,7 @@
     </row>
     <row r="122" hidden="true">
       <c r="A122" t="s" s="2">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B122" t="s" s="2">
         <v>564</v>
@@ -17256,7 +17255,7 @@
     </row>
     <row r="123" hidden="true">
       <c r="A123" t="s" s="2">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B123" t="s" s="2">
         <v>514</v>
@@ -17376,7 +17375,7 @@
     </row>
     <row r="124" hidden="true">
       <c r="A124" t="s" s="2">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B124" t="s" s="2">
         <v>514</v>
@@ -17500,7 +17499,7 @@
     </row>
     <row r="125" hidden="true">
       <c r="A125" t="s" s="2">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B125" t="s" s="2">
         <v>568</v>
@@ -17618,7 +17617,7 @@
     </row>
     <row r="126" hidden="true">
       <c r="A126" t="s" s="2">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B126" t="s" s="2">
         <v>570</v>
@@ -17738,7 +17737,7 @@
     </row>
     <row r="127" hidden="true">
       <c r="A127" t="s" s="2">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B127" t="s" s="2">
         <v>572</v>
@@ -17860,7 +17859,7 @@
     </row>
     <row r="128" hidden="true">
       <c r="A128" t="s" s="2">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B128" t="s" s="2">
         <v>582</v>
@@ -17984,7 +17983,7 @@
     </row>
     <row r="129" hidden="true">
       <c r="A129" t="s" s="2">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B129" t="s" s="2">
         <v>593</v>
@@ -18106,7 +18105,7 @@
     </row>
     <row r="130" hidden="true">
       <c r="A130" t="s" s="2">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B130" t="s" s="2">
         <v>601</v>
@@ -18228,7 +18227,7 @@
     </row>
     <row r="131" hidden="true">
       <c r="A131" t="s" s="2">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B131" t="s" s="2">
         <v>611</v>
@@ -18350,7 +18349,7 @@
     </row>
     <row r="132" hidden="true">
       <c r="A132" t="s" s="2">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B132" t="s" s="2">
         <v>522</v>
@@ -18472,7 +18471,7 @@
     </row>
     <row r="133" hidden="true">
       <c r="A133" t="s" s="2">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B133" t="s" s="2">
         <v>527</v>
@@ -18537,9 +18536,11 @@
       <c r="X133" t="s" s="2">
         <v>257</v>
       </c>
-      <c r="Y133" s="2"/>
+      <c r="Y133" t="s" s="2">
+        <v>375</v>
+      </c>
       <c r="Z133" t="s" s="2">
-        <v>620</v>
+        <v>376</v>
       </c>
       <c r="AA133" t="s" s="2">
         <v>38</v>
@@ -18592,7 +18593,7 @@
     </row>
     <row r="134" hidden="true">
       <c r="A134" t="s" s="2">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B134" t="s" s="2">
         <v>528</v>
@@ -18714,13 +18715,13 @@
     </row>
     <row r="135" hidden="true">
       <c r="A135" t="s" s="2">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B135" t="s" s="2">
         <v>496</v>
       </c>
       <c r="C135" t="s" s="2">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="D135" t="s" s="2">
         <v>38</v>
@@ -18745,10 +18746,10 @@
         <v>426</v>
       </c>
       <c r="L135" t="s" s="2">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="M135" t="s" s="2">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="N135" t="s" s="2">
         <v>499</v>
@@ -18838,7 +18839,7 @@
     </row>
     <row r="136" hidden="true">
       <c r="A136" t="s" s="2">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B136" t="s" s="2">
         <v>505</v>
@@ -18956,7 +18957,7 @@
     </row>
     <row r="137" hidden="true">
       <c r="A137" t="s" s="2">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B137" t="s" s="2">
         <v>506</v>
@@ -19076,7 +19077,7 @@
     </row>
     <row r="138" hidden="true">
       <c r="A138" t="s" s="2">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B138" t="s" s="2">
         <v>507</v>
@@ -19198,7 +19199,7 @@
     </row>
     <row r="139" hidden="true">
       <c r="A139" t="s" s="2">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B139" t="s" s="2">
         <v>508</v>
@@ -19320,7 +19321,7 @@
     </row>
     <row r="140" hidden="true">
       <c r="A140" t="s" s="2">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B140" t="s" s="2">
         <v>539</v>
@@ -19438,7 +19439,7 @@
     </row>
     <row r="141" hidden="true">
       <c r="A141" t="s" s="2">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B141" t="s" s="2">
         <v>541</v>
@@ -19558,7 +19559,7 @@
     </row>
     <row r="142" hidden="true">
       <c r="A142" t="s" s="2">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B142" t="s" s="2">
         <v>543</v>
@@ -19678,13 +19679,13 @@
     </row>
     <row r="143" hidden="true">
       <c r="A143" t="s" s="2">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B143" t="s" s="2">
         <v>543</v>
       </c>
       <c r="C143" t="s" s="2">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="D143" t="s" s="2">
         <v>38</v>
@@ -19802,7 +19803,7 @@
     </row>
     <row r="144" hidden="true">
       <c r="A144" t="s" s="2">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B144" t="s" s="2">
         <v>549</v>
@@ -19920,7 +19921,7 @@
     </row>
     <row r="145" hidden="true">
       <c r="A145" t="s" s="2">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B145" t="s" s="2">
         <v>551</v>
@@ -20040,7 +20041,7 @@
     </row>
     <row r="146" hidden="true">
       <c r="A146" t="s" s="2">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B146" t="s" s="2">
         <v>553</v>
@@ -20162,7 +20163,7 @@
     </row>
     <row r="147" hidden="true">
       <c r="A147" t="s" s="2">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B147" t="s" s="2">
         <v>555</v>
@@ -20282,7 +20283,7 @@
     </row>
     <row r="148" hidden="true">
       <c r="A148" t="s" s="2">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B148" t="s" s="2">
         <v>557</v>
@@ -20311,10 +20312,10 @@
         <v>72</v>
       </c>
       <c r="L148" t="s" s="2">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="M148" t="s" s="2">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="N148" t="s" s="2">
         <v>218</v>
@@ -20327,7 +20328,7 @@
       </c>
       <c r="Q148" s="2"/>
       <c r="R148" t="s" s="2">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="S148" t="s" s="2">
         <v>38</v>
@@ -20404,7 +20405,7 @@
     </row>
     <row r="149" hidden="true">
       <c r="A149" t="s" s="2">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B149" t="s" s="2">
         <v>560</v>
@@ -20526,7 +20527,7 @@
     </row>
     <row r="150" hidden="true">
       <c r="A150" t="s" s="2">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B150" t="s" s="2">
         <v>562</v>
@@ -20648,7 +20649,7 @@
     </row>
     <row r="151" hidden="true">
       <c r="A151" t="s" s="2">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B151" t="s" s="2">
         <v>564</v>
@@ -20770,7 +20771,7 @@
     </row>
     <row r="152" hidden="true">
       <c r="A152" t="s" s="2">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B152" t="s" s="2">
         <v>514</v>
@@ -20892,7 +20893,7 @@
     </row>
     <row r="153" hidden="true">
       <c r="A153" t="s" s="2">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B153" t="s" s="2">
         <v>522</v>
@@ -21014,7 +21015,7 @@
     </row>
     <row r="154" hidden="true">
       <c r="A154" t="s" s="2">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="B154" t="s" s="2">
         <v>527</v>
@@ -21079,9 +21080,11 @@
       <c r="X154" t="s" s="2">
         <v>257</v>
       </c>
-      <c r="Y154" s="2"/>
+      <c r="Y154" t="s" s="2">
+        <v>375</v>
+      </c>
       <c r="Z154" t="s" s="2">
-        <v>620</v>
+        <v>376</v>
       </c>
       <c r="AA154" t="s" s="2">
         <v>38</v>
@@ -21134,7 +21137,7 @@
     </row>
     <row r="155" hidden="true">
       <c r="A155" t="s" s="2">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B155" t="s" s="2">
         <v>528</v>

</xml_diff>